<commit_message>
commit #3 - bug fix
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yakuz\OneDrive\Documents\UiPath\Performer_IE6_SelectAmazonProduct_Process\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CA4603-EC02-4112-86FF-D0A9DF683775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76946F93-1885-4589-B946-62A2AF164510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9912" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="9912" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -18,16 +18,11 @@
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="75">
   <si>
     <t>Name</t>
   </si>
@@ -176,9 +171,6 @@
     <t>BrowserType</t>
   </si>
   <si>
-    <t>ProductSearchQueue</t>
-  </si>
-  <si>
     <t>(empty)</t>
   </si>
   <si>
@@ -194,9 +186,6 @@
     <t>Amazon_Password</t>
   </si>
   <si>
-    <t>Chrome</t>
-  </si>
-  <si>
     <t>https://www.amazon.co.uk</t>
   </si>
   <si>
@@ -240,6 +229,24 @@
   </si>
   <si>
     <t>Browser to use</t>
+  </si>
+  <si>
+    <t>IE6_AmazonScrape_Keywords</t>
+  </si>
+  <si>
+    <t>Edge</t>
+  </si>
+  <si>
+    <t>logF_BusinessProcessName</t>
+  </si>
+  <si>
+    <t>AmazonProductSearch</t>
+  </si>
+  <si>
+    <t>Process name added to all log entries</t>
+  </si>
+  <si>
+    <t>nikpirat2@gmail.com's workspace</t>
   </si>
 </sst>
 </file>
@@ -299,10 +306,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -311,7 +318,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -336,9 +343,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -376,7 +383,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -482,7 +489,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -624,7 +631,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -680,21 +687,21 @@
         <v>38</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.4">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>50</v>
+      <c r="B3" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -705,7 +712,7 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.4">
@@ -716,7 +723,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
@@ -724,10 +731,10 @@
         <v>39</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
@@ -738,7 +745,7 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -749,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
@@ -757,10 +764,10 @@
         <v>42</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
@@ -768,10 +775,10 @@
         <v>43</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -779,10 +786,10 @@
         <v>44</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
@@ -790,10 +797,10 @@
         <v>45</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -801,10 +808,10 @@
         <v>46</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
@@ -815,7 +822,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -823,13 +830,23 @@
         <v>48</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" t="s">
+        <v>73</v>
+      </c>
+    </row>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
@@ -1816,9 +1833,10 @@
   <phoneticPr fontId="2"/>
   <hyperlinks>
     <hyperlink ref="B6" r:id="rId1" xr:uid="{F67F8771-856C-4625-93AE-C4C7C9C44C86}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{52DE5A8D-E47B-43A8-BC55-8B5EC000F398}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>